<commit_message>
feat: stabilize v2 excel db reporting loop
</commit_message>
<xml_diff>
--- a/samples/ai_construction_weekly_report.xlsx
+++ b/samples/ai_construction_weekly_report.xlsx
@@ -53,7 +53,7 @@
     <t>위험공종</t>
   </si>
   <si>
-    <t>civil</t>
+    <t>토목</t>
   </si>
   <si>
     <t>핵심 리스크</t>
@@ -86,7 +86,7 @@
     <t>Normal concrete curing</t>
   </si>
   <si>
-    <t>architecture</t>
+    <t>건축</t>
   </si>
   <si>
     <t>1F</t>
@@ -122,7 +122,7 @@
     <t>MEP ceiling framing cost overrun</t>
   </si>
   <si>
-    <t>mechanical</t>
+    <t>기계설비</t>
   </si>
   <si>
     <t>2F</t>
@@ -137,7 +137,7 @@
     <t>Fire pump delivery delay</t>
   </si>
   <si>
-    <t>fire_protection</t>
+    <t>소방설비</t>
   </si>
   <si>
     <t>Machine Room</t>
@@ -152,7 +152,7 @@
     <t>Electrical panel inspection delay</t>
   </si>
   <si>
-    <t>electrical</t>
+    <t>전기설비</t>
   </si>
   <si>
     <t>EPS</t>

</xml_diff>

<commit_message>
feat: stabilize construction scheduler v2.1
</commit_message>
<xml_diff>
--- a/samples/ai_construction_weekly_report.xlsx
+++ b/samples/ai_construction_weekly_report.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="108">
   <si>
     <t>현장소장 대시보드</t>
   </si>
@@ -62,6 +62,12 @@
     <t>원가 과투입 검토 필요</t>
   </si>
   <si>
+    <t>종합 의견</t>
+  </si>
+  <si>
+    <t>계획 62.0% 대비 실적 39.0%로 차이 -23.0%입니다. 부진공정 5건은 즉시 조치 필요하며 담당자 확인 필요.</t>
+  </si>
+  <si>
     <t>activity_id</t>
   </si>
   <si>
@@ -179,28 +185,28 @@
     <t>Lee</t>
   </si>
   <si>
-    <t>Delayed rebar assembly progress delay: planned 80.0%, actual 55.0%, gap 25.0%.</t>
+    <t>Delayed rebar assembly: Delayed rebar assembly progress delay: planned 80.0%, actual 55.0%, gap 25.0%. 담당자 확인 필요.</t>
   </si>
   <si>
     <t>Park</t>
   </si>
   <si>
-    <t>Concrete pour blocked by predecessor progress delay: planned 30.0%, actual 0.0%, gap 30.0%.</t>
+    <t>Concrete pour blocked by predecessor: Concrete pour blocked by predecessor progress delay: planned 30.0%, actual 0.0%, gap 30.0%. 담당자 확인 필요.</t>
   </si>
   <si>
     <t>Choi</t>
   </si>
   <si>
-    <t>MEP ceiling framing cost overrun progress delay: planned 60.0%, actual 45.0%, gap 15.0%.</t>
+    <t>MEP ceiling framing cost overrun: MEP ceiling framing cost overrun progress delay: planned 60.0%, actual 45.0%, gap 15.0%. 담당자 확인 필요.</t>
   </si>
   <si>
     <t>Jung</t>
   </si>
   <si>
-    <t>Fire pump delivery delay progress delay: planned 40.0%, actual 0.0%, gap 40.0%.</t>
-  </si>
-  <si>
-    <t>Electrical panel inspection delay progress delay: planned 70.0%, actual 40.0%, gap 30.0%.</t>
+    <t>Fire pump delivery delay: Fire pump delivery delay progress delay: planned 40.0%, actual 0.0%, gap 40.0%. 담당자 확인 필요.</t>
+  </si>
+  <si>
+    <t>Electrical panel inspection delay: Electrical panel inspection delay progress delay: planned 70.0%, actual 40.0%, gap 30.0%. 담당자 확인 필요.</t>
   </si>
   <si>
     <t>candidate</t>
@@ -218,24 +224,7 @@
     <t>검토 필요</t>
   </si>
   <si>
-    <t>Delayed rebar assembly 지연 원인(schedule_progress_delay)에 대한 만회대책 초안입니다. 검토 필요.
-1. 현장 협의 후보: 담당자, 협력사, 감리와 원인 및 만회 가능 조건을 검토하는 초안입니다. 검토 필요.</t>
-  </si>
-  <si>
-    <t>Concrete pour blocked by predecessor 지연 원인(schedule_progress_delay)에 대한 만회대책 초안입니다. 검토 필요.
-1. 현장 협의 후보: 담당자, 협력사, 감리와 원인 및 만회 가능 조건을 검토하는 초안입니다. 검토 필요.</t>
-  </si>
-  <si>
-    <t>MEP ceiling framing cost overrun 지연 원인(schedule_progress_delay)에 대한 만회대책 초안입니다. 검토 필요.
-1. 현장 협의 후보: 담당자, 협력사, 감리와 원인 및 만회 가능 조건을 검토하는 초안입니다. 검토 필요.</t>
-  </si>
-  <si>
-    <t>Fire pump delivery delay 지연 원인(schedule_progress_delay)에 대한 만회대책 초안입니다. 검토 필요.
-1. 현장 협의 후보: 담당자, 협력사, 감리와 원인 및 만회 가능 조건을 검토하는 초안입니다. 검토 필요.</t>
-  </si>
-  <si>
-    <t>Electrical panel inspection delay 지연 원인(schedule_progress_delay)에 대한 만회대책 초안입니다. 검토 필요.
-1. 현장 협의 후보: 담당자, 협력사, 감리와 원인 및 만회 가능 조건을 검토하는 초안입니다. 검토 필요.</t>
+    <t>현장 협의 후보: 검토 필요 현장소장 승인 후 시행 검토 필요.</t>
   </si>
   <si>
     <t>progress_pct</t>
@@ -343,7 +332,7 @@
     <t>report_style</t>
   </si>
   <si>
-    <t>weekly_meeting</t>
+    <t>internal</t>
   </si>
   <si>
     <t>delayed_activity_count</t>
@@ -740,7 +729,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -818,6 +807,14 @@
       </c>
       <c r="B10" t="s">
         <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -832,39 +829,39 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F2">
         <v>100</v>
@@ -872,19 +869,19 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C3" t="s">
         <v>10</v>
       </c>
       <c r="D3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F3">
         <v>55</v>
@@ -892,19 +889,19 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C4" t="s">
         <v>10</v>
       </c>
       <c r="D4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E4" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F4">
         <v>0</v>
@@ -912,19 +909,19 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F5">
         <v>45</v>
@@ -932,19 +929,19 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F6">
         <v>0</v>
@@ -952,19 +949,19 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B7" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D7" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E7" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F7">
         <v>40</v>
@@ -982,156 +979,156 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="G2" s="3">
         <v>33</v>
       </c>
       <c r="H2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G3" s="3">
         <v>38</v>
       </c>
       <c r="H3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="G4" s="3">
         <v>15</v>
       </c>
       <c r="H4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G5" s="3">
         <v>51</v>
       </c>
       <c r="H5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F6" s="3"/>
       <c r="G6" s="3">
         <v>44</v>
       </c>
       <c r="H6" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -1146,79 +1143,79 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F4" t="s">
         <v>67</v>
@@ -1226,42 +1223,42 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -1276,36 +1273,36 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>73</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C2" s="3">
         <v>45</v>
@@ -1338,121 +1335,121 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C3" t="s">
         <v>10</v>
       </c>
       <c r="D3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C4" t="s">
         <v>10</v>
       </c>
       <c r="D4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E4" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E6" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B7" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D7" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E7" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -1467,39 +1464,39 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>85</v>
-      </c>
       <c r="F1" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E2" t="s">
         <v>86</v>
-      </c>
-      <c r="D2" t="s">
-        <v>87</v>
-      </c>
-      <c r="E2" t="s">
-        <v>88</v>
       </c>
       <c r="F2">
         <v>100</v>
@@ -1507,19 +1504,19 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D3" t="s">
+        <v>88</v>
+      </c>
+      <c r="E3" t="s">
         <v>89</v>
-      </c>
-      <c r="D3" t="s">
-        <v>90</v>
-      </c>
-      <c r="E3" t="s">
-        <v>91</v>
       </c>
       <c r="F3">
         <v>55</v>
@@ -1527,19 +1524,19 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C4" t="s">
+        <v>90</v>
+      </c>
+      <c r="D4" t="s">
+        <v>91</v>
+      </c>
+      <c r="E4" t="s">
         <v>92</v>
-      </c>
-      <c r="D4" t="s">
-        <v>93</v>
-      </c>
-      <c r="E4" t="s">
-        <v>94</v>
       </c>
       <c r="F4">
         <v>0</v>
@@ -1547,19 +1544,19 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C5" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D5" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F5">
         <v>45</v>
@@ -1567,19 +1564,19 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D6" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="E6" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F6">
         <v>0</v>
@@ -1587,19 +1584,19 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B7" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C7" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D7" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E7" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F7">
         <v>40</v>
@@ -1617,28 +1614,36 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" s="2" t="s">
+      <c r="A3" t="s">
         <v>102</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>104</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>105</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B5">
         <v>5</v>
@@ -1646,7 +1651,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B6">
         <v>5</v>
@@ -1654,10 +1659,10 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B7" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: harden construction scheduler v2.2 field import
</commit_message>
<xml_diff>
--- a/samples/ai_construction_weekly_report.xlsx
+++ b/samples/ai_construction_weekly_report.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="113">
   <si>
     <t>현장소장 대시보드</t>
   </si>
@@ -240,6 +240,21 @@
   </si>
   <si>
     <t>billing_rate</t>
+  </si>
+  <si>
+    <t>planned_value</t>
+  </si>
+  <si>
+    <t>earned_value</t>
+  </si>
+  <si>
+    <t>actual_cost</t>
+  </si>
+  <si>
+    <t>spi</t>
+  </si>
+  <si>
+    <t>cpi</t>
   </si>
   <si>
     <t>overrun</t>
@@ -1268,10 +1283,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:13">
       <c r="A1" s="2" t="s">
         <v>15</v>
       </c>
@@ -1296,8 +1311,23 @@
       <c r="H1" s="2" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="2" spans="1:8">
+      <c r="I1" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
       <c r="A2" s="3" t="s">
         <v>33</v>
       </c>
@@ -1319,7 +1349,22 @@
       <c r="G2" s="3">
         <v>38.46</v>
       </c>
-      <c r="H2" s="3" t="b">
+      <c r="H2" s="3">
+        <v>600</v>
+      </c>
+      <c r="I2" s="3">
+        <v>450</v>
+      </c>
+      <c r="J2" s="3">
+        <v>720</v>
+      </c>
+      <c r="K2" s="3">
+        <v>0.75</v>
+      </c>
+      <c r="L2" s="3">
+        <v>0.62</v>
+      </c>
+      <c r="M2" s="3" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1347,7 +1392,7 @@
         <v>18</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -1364,7 +1409,7 @@
         <v>24</v>
       </c>
       <c r="E2" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -1381,7 +1426,7 @@
         <v>28</v>
       </c>
       <c r="E3" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -1398,7 +1443,7 @@
         <v>28</v>
       </c>
       <c r="E4" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -1415,7 +1460,7 @@
         <v>36</v>
       </c>
       <c r="E5" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -1432,7 +1477,7 @@
         <v>41</v>
       </c>
       <c r="E6" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -1449,7 +1494,7 @@
         <v>46</v>
       </c>
       <c r="E7" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -1470,13 +1515,13 @@
         <v>16</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>20</v>
@@ -1490,13 +1535,13 @@
         <v>22</v>
       </c>
       <c r="C2" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="D2" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="E2" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="F2">
         <v>100</v>
@@ -1510,13 +1555,13 @@
         <v>27</v>
       </c>
       <c r="C3" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="D3" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="E3" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="F3">
         <v>55</v>
@@ -1530,13 +1575,13 @@
         <v>31</v>
       </c>
       <c r="C4" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="D4" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="E4" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="F4">
         <v>0</v>
@@ -1550,13 +1595,13 @@
         <v>34</v>
       </c>
       <c r="C5" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D5" t="s">
+        <v>99</v>
+      </c>
+      <c r="E5" t="s">
         <v>94</v>
-      </c>
-      <c r="E5" t="s">
-        <v>89</v>
       </c>
       <c r="F5">
         <v>45</v>
@@ -1570,13 +1615,13 @@
         <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="D6" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="E6" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="F6">
         <v>0</v>
@@ -1590,13 +1635,13 @@
         <v>44</v>
       </c>
       <c r="C7" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="D7" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="E7" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="F7">
         <v>40</v>
@@ -1614,23 +1659,23 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="B3" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -1643,7 +1688,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="B5">
         <v>5</v>
@@ -1651,7 +1696,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="B6">
         <v>5</v>
@@ -1659,10 +1704,10 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="B7" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>